<commit_message>
Update quiz result messages for different score ranges
Modify results page logic and templates to display conditional messages based on user score: "We see you! Stop flexing now!" for scores >= 7, and "Not enough knowledge to flex" for scores < 7. Also, change "Good Try!" to "Bravo!" for scores below 7.

Replit-Commit-Author: Agent
Replit-Commit-Session-Id: 37877615-d133-4c1f-b6b6-f54cbc6b3767
Replit-Commit-Checkpoint-Type: full_checkpoint
Replit-Commit-Screenshot-Url: https://storage.googleapis.com/screenshot-production-us-central1/474f6d33-5530-4c51-8e53-e2d7cdb3d75e/37877615-d133-4c1f-b6b6-f54cbc6b3767/xbl3oAo
</commit_message>
<xml_diff>
--- a/quiz_results.xlsx
+++ b/quiz_results.xlsx
@@ -426,10 +426,10 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G3"/>
+  <dimension ref="A1:G4"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="7" customWidth="1" min="1" max="1"/>
+    <col width="8" customWidth="1" min="1" max="1"/>
     <col width="8" customWidth="1" min="2" max="2"/>
     <col width="10" customWidth="1" min="3" max="3"/>
     <col width="7" customWidth="1" min="4" max="4"/>
@@ -549,6 +549,43 @@
         </is>
       </c>
     </row>
+    <row r="4">
+      <c r="A4" t="inlineStr">
+        <is>
+          <t>labubu</t>
+        </is>
+      </c>
+      <c r="B4" t="inlineStr">
+        <is>
+          <t>123456</t>
+        </is>
+      </c>
+      <c r="C4" t="inlineStr">
+        <is>
+          <t>****9012</t>
+        </is>
+      </c>
+      <c r="D4" t="inlineStr">
+        <is>
+          <t>1/10</t>
+        </is>
+      </c>
+      <c r="E4" t="inlineStr">
+        <is>
+          <t>10.00%</t>
+        </is>
+      </c>
+      <c r="F4" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="G4" t="inlineStr">
+        <is>
+          <t>2025-10-22 09:22:27</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Adjust quiz feedback based on user scores
Update quiz result messages and feedback strings for low (below 7) and high (7+) scores.

Replit-Commit-Author: Agent
Replit-Commit-Session-Id: 37877615-d133-4c1f-b6b6-f54cbc6b3767
Replit-Commit-Checkpoint-Type: full_checkpoint
Replit-Commit-Screenshot-Url: https://storage.googleapis.com/screenshot-production-us-central1/474f6d33-5530-4c51-8e53-e2d7cdb3d75e/37877615-d133-4c1f-b6b6-f54cbc6b3767/xbl3oAo
</commit_message>
<xml_diff>
--- a/quiz_results.xlsx
+++ b/quiz_results.xlsx
@@ -426,7 +426,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G4"/>
+  <dimension ref="A1:G5"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="8" customWidth="1" min="1" max="1"/>
@@ -586,6 +586,43 @@
         </is>
       </c>
     </row>
+    <row r="5">
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>daulat</t>
+        </is>
+      </c>
+      <c r="B5" t="inlineStr">
+        <is>
+          <t>123456</t>
+        </is>
+      </c>
+      <c r="C5" t="inlineStr">
+        <is>
+          <t>****9012</t>
+        </is>
+      </c>
+      <c r="D5" t="inlineStr">
+        <is>
+          <t>3/10</t>
+        </is>
+      </c>
+      <c r="E5" t="inlineStr">
+        <is>
+          <t>30.00%</t>
+        </is>
+      </c>
+      <c r="F5" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="G5" t="inlineStr">
+        <is>
+          <t>2025-10-22 09:30:23</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Update quiz interface and submission logic for improved user experience
Update answer selection glow to blue, enable submit button on last question, and adjust carousel height in `quiz.html` and `static/main.js`.

Replit-Commit-Author: Agent
Replit-Commit-Session-Id: 37877615-d133-4c1f-b6b6-f54cbc6b3767
Replit-Commit-Checkpoint-Type: full_checkpoint
Replit-Commit-Screenshot-Url: https://storage.googleapis.com/screenshot-production-us-central1/474f6d33-5530-4c51-8e53-e2d7cdb3d75e/37877615-d133-4c1f-b6b6-f54cbc6b3767/boTbOo7
</commit_message>
<xml_diff>
--- a/quiz_results.xlsx
+++ b/quiz_results.xlsx
@@ -426,7 +426,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G5"/>
+  <dimension ref="A1:G6"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="8" customWidth="1" min="1" max="1"/>
@@ -623,6 +623,43 @@
         </is>
       </c>
     </row>
+    <row r="6">
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>abc</t>
+        </is>
+      </c>
+      <c r="B6" t="inlineStr">
+        <is>
+          <t>123456</t>
+        </is>
+      </c>
+      <c r="C6" t="inlineStr">
+        <is>
+          <t>****8912</t>
+        </is>
+      </c>
+      <c r="D6" t="inlineStr">
+        <is>
+          <t>3/10</t>
+        </is>
+      </c>
+      <c r="E6" t="inlineStr">
+        <is>
+          <t>30.00%</t>
+        </is>
+      </c>
+      <c r="F6" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="G6" t="inlineStr">
+        <is>
+          <t>2025-10-22 09:49:38</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Update result page to display score and participant name
Changes the title from "Results" to "Score" in result.html and retrieves the participant's name to display alongside their score in app.py.

Replit-Commit-Author: Agent
Replit-Commit-Session-Id: 37877615-d133-4c1f-b6b6-f54cbc6b3767
Replit-Commit-Checkpoint-Type: full_checkpoint
Replit-Commit-Screenshot-Url: https://storage.googleapis.com/screenshot-production-us-central1/474f6d33-5530-4c51-8e53-e2d7cdb3d75e/37877615-d133-4c1f-b6b6-f54cbc6b3767/iS1H8wd
</commit_message>
<xml_diff>
--- a/quiz_results.xlsx
+++ b/quiz_results.xlsx
@@ -426,7 +426,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G6"/>
+  <dimension ref="A1:G7"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="8" customWidth="1" min="1" max="1"/>
@@ -660,6 +660,43 @@
         </is>
       </c>
     </row>
+    <row r="7">
+      <c r="A7" t="inlineStr">
+        <is>
+          <t>Arshae</t>
+        </is>
+      </c>
+      <c r="B7" t="inlineStr">
+        <is>
+          <t>123456</t>
+        </is>
+      </c>
+      <c r="C7" t="inlineStr">
+        <is>
+          <t>****9012</t>
+        </is>
+      </c>
+      <c r="D7" t="inlineStr">
+        <is>
+          <t>3/10</t>
+        </is>
+      </c>
+      <c r="E7" t="inlineStr">
+        <is>
+          <t>30.00%</t>
+        </is>
+      </c>
+      <c r="F7" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="G7" t="inlineStr">
+        <is>
+          <t>2025-10-22 09:59:47</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Update the quiz timer to last for 100 seconds
Adjusted the `timeRemaining` variable in `static/main.js` and the displayed timer count in `templates/quiz.html` from 80 to 100 seconds.

Replit-Commit-Author: Agent
Replit-Commit-Session-Id: 37877615-d133-4c1f-b6b6-f54cbc6b3767
Replit-Commit-Checkpoint-Type: full_checkpoint
Replit-Commit-Screenshot-Url: https://storage.googleapis.com/screenshot-production-us-central1/474f6d33-5530-4c51-8e53-e2d7cdb3d75e/37877615-d133-4c1f-b6b6-f54cbc6b3767/GhOecdf
</commit_message>
<xml_diff>
--- a/quiz_results.xlsx
+++ b/quiz_results.xlsx
@@ -426,7 +426,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G2"/>
+  <dimension ref="A1:G4"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="11" customWidth="1" min="1" max="1"/>
@@ -512,6 +512,80 @@
         </is>
       </c>
     </row>
+    <row r="3">
+      <c r="A3" t="inlineStr">
+        <is>
+          <t>PS</t>
+        </is>
+      </c>
+      <c r="B3" t="inlineStr">
+        <is>
+          <t>123456</t>
+        </is>
+      </c>
+      <c r="C3" t="inlineStr">
+        <is>
+          <t>****9012</t>
+        </is>
+      </c>
+      <c r="D3" t="inlineStr">
+        <is>
+          <t>2/10</t>
+        </is>
+      </c>
+      <c r="E3" t="inlineStr">
+        <is>
+          <t>20.00%</t>
+        </is>
+      </c>
+      <c r="F3" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="G3" t="inlineStr">
+        <is>
+          <t>2025-10-22 10:26:22</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="inlineStr">
+        <is>
+          <t>Emon</t>
+        </is>
+      </c>
+      <c r="B4" t="inlineStr">
+        <is>
+          <t>012345</t>
+        </is>
+      </c>
+      <c r="C4" t="inlineStr">
+        <is>
+          <t>02</t>
+        </is>
+      </c>
+      <c r="D4" t="inlineStr">
+        <is>
+          <t>5/10</t>
+        </is>
+      </c>
+      <c r="E4" t="inlineStr">
+        <is>
+          <t>50.00%</t>
+        </is>
+      </c>
+      <c r="F4" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="G4" t="inlineStr">
+        <is>
+          <t>2025-10-22 10:29:21</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Adjust spacing and sizing for the quiz results page
Reduces the size of the score circle, result card, and associated text elements on the results page to improve layout and spacing. Adjusts SVG dimensions and circle properties for the score visualization. Updates padding, margins, and font sizes across various result page components.

Replit-Commit-Author: Agent
Replit-Commit-Session-Id: 37877615-d133-4c1f-b6b6-f54cbc6b3767
Replit-Commit-Checkpoint-Type: full_checkpoint
Replit-Commit-Screenshot-Url: https://storage.googleapis.com/screenshot-production-us-central1/474f6d33-5530-4c51-8e53-e2d7cdb3d75e/37877615-d133-4c1f-b6b6-f54cbc6b3767/WtpoTww
</commit_message>
<xml_diff>
--- a/quiz_results.xlsx
+++ b/quiz_results.xlsx
@@ -426,10 +426,10 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G4"/>
+  <dimension ref="A1:G7"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="11" customWidth="1" min="1" max="1"/>
+    <col width="15" customWidth="1" min="1" max="1"/>
     <col width="8" customWidth="1" min="2" max="2"/>
     <col width="10" customWidth="1" min="3" max="3"/>
     <col width="7" customWidth="1" min="4" max="4"/>
@@ -586,6 +586,117 @@
         </is>
       </c>
     </row>
+    <row r="5">
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>abc</t>
+        </is>
+      </c>
+      <c r="B5" t="inlineStr">
+        <is>
+          <t>123456</t>
+        </is>
+      </c>
+      <c r="C5" t="inlineStr">
+        <is>
+          <t>****9012</t>
+        </is>
+      </c>
+      <c r="D5" t="inlineStr">
+        <is>
+          <t>7/10</t>
+        </is>
+      </c>
+      <c r="E5" t="inlineStr">
+        <is>
+          <t>70.00%</t>
+        </is>
+      </c>
+      <c r="F5" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="G5" t="inlineStr">
+        <is>
+          <t>2025-10-22 10:43:04</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>ayon</t>
+        </is>
+      </c>
+      <c r="B6" t="inlineStr">
+        <is>
+          <t>123456</t>
+        </is>
+      </c>
+      <c r="C6" t="inlineStr">
+        <is>
+          <t>****9012</t>
+        </is>
+      </c>
+      <c r="D6" t="inlineStr">
+        <is>
+          <t>7/10</t>
+        </is>
+      </c>
+      <c r="E6" t="inlineStr">
+        <is>
+          <t>70.00%</t>
+        </is>
+      </c>
+      <c r="F6" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="G6" t="inlineStr">
+        <is>
+          <t>2025-10-22 10:46:54</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="inlineStr">
+        <is>
+          <t>Kaji the paji</t>
+        </is>
+      </c>
+      <c r="B7" t="inlineStr">
+        <is>
+          <t>123456</t>
+        </is>
+      </c>
+      <c r="C7" t="inlineStr">
+        <is>
+          <t>****test</t>
+        </is>
+      </c>
+      <c r="D7" t="inlineStr">
+        <is>
+          <t>10/10</t>
+        </is>
+      </c>
+      <c r="E7" t="inlineStr">
+        <is>
+          <t>100.00%</t>
+        </is>
+      </c>
+      <c r="F7" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="G7" t="inlineStr">
+        <is>
+          <t>2025-10-22 10:52:29</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Adjust spacing on the final quiz results page
No code changes detected. The diff only contains metadata for the file quiz_results.xlsx.

Replit-Commit-Author: Agent
Replit-Commit-Session-Id: 37877615-d133-4c1f-b6b6-f54cbc6b3767
Replit-Commit-Checkpoint-Type: full_checkpoint
Replit-Commit-Screenshot-Url: https://storage.googleapis.com/screenshot-production-us-central1/474f6d33-5530-4c51-8e53-e2d7cdb3d75e/37877615-d133-4c1f-b6b6-f54cbc6b3767/WtpoTww
</commit_message>
<xml_diff>
--- a/quiz_results.xlsx
+++ b/quiz_results.xlsx
@@ -426,7 +426,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G7"/>
+  <dimension ref="A1:G8"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="15" customWidth="1" min="1" max="1"/>
@@ -697,6 +697,43 @@
         </is>
       </c>
     </row>
+    <row r="8">
+      <c r="A8" t="inlineStr">
+        <is>
+          <t>abc</t>
+        </is>
+      </c>
+      <c r="B8" t="inlineStr">
+        <is>
+          <t>123456</t>
+        </is>
+      </c>
+      <c r="C8" t="inlineStr">
+        <is>
+          <t>****9012</t>
+        </is>
+      </c>
+      <c r="D8" t="inlineStr">
+        <is>
+          <t>0/10</t>
+        </is>
+      </c>
+      <c r="E8" t="inlineStr">
+        <is>
+          <t>0.00%</t>
+        </is>
+      </c>
+      <c r="F8" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="G8" t="inlineStr">
+        <is>
+          <t>2025-10-22 11:18:41</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Remove explicit previous and next navigation buttons from quiz flow
Removes HTML elements and JavaScript event listeners for previous/next buttons, and modifies `updateNavButtons` function to hide next button and disable previous button based on current question index, aligning with swipe-based navigation.

Replit-Commit-Author: Agent
Replit-Commit-Session-Id: 37877615-d133-4c1f-b6b6-f54cbc6b3767
Replit-Commit-Checkpoint-Type: full_checkpoint
Replit-Commit-Screenshot-Url: https://storage.googleapis.com/screenshot-production-us-central1/474f6d33-5530-4c51-8e53-e2d7cdb3d75e/37877615-d133-4c1f-b6b6-f54cbc6b3767/vU7O0Iz
</commit_message>
<xml_diff>
--- a/quiz_results.xlsx
+++ b/quiz_results.xlsx
@@ -426,10 +426,10 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G2"/>
+  <dimension ref="A1:G3"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="7" customWidth="1" min="1" max="1"/>
+    <col width="15" customWidth="1" min="1" max="1"/>
     <col width="8" customWidth="1" min="2" max="2"/>
     <col width="10" customWidth="1" min="3" max="3"/>
     <col width="7" customWidth="1" min="4" max="4"/>
@@ -512,6 +512,43 @@
         </is>
       </c>
     </row>
+    <row r="3">
+      <c r="A3" t="inlineStr">
+        <is>
+          <t>Player-123456</t>
+        </is>
+      </c>
+      <c r="B3" t="inlineStr">
+        <is>
+          <t>123456</t>
+        </is>
+      </c>
+      <c r="C3" t="inlineStr">
+        <is>
+          <t>****3456</t>
+        </is>
+      </c>
+      <c r="D3" t="inlineStr">
+        <is>
+          <t>0/10</t>
+        </is>
+      </c>
+      <c r="E3" t="inlineStr">
+        <is>
+          <t>0.00%</t>
+        </is>
+      </c>
+      <c r="F3" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="G3" t="inlineStr">
+        <is>
+          <t>2025-10-29 04:52:25</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Update progress bar and dots to reflect answered questions
Modify `static/main.js` and `templates/quiz.html` to correctly update the progress bar width and dot appearance based on the number of answered questions, ensuring the progress bar aligns with the visual stamps as requested.

Replit-Commit-Author: Agent
Replit-Commit-Session-Id: 37877615-d133-4c1f-b6b6-f54cbc6b3767
Replit-Commit-Checkpoint-Type: full_checkpoint
Replit-Commit-Screenshot-Url: https://storage.googleapis.com/screenshot-production-us-central1/474f6d33-5530-4c51-8e53-e2d7cdb3d75e/37877615-d133-4c1f-b6b6-f54cbc6b3767/jRkhkXk
</commit_message>
<xml_diff>
--- a/quiz_results.xlsx
+++ b/quiz_results.xlsx
@@ -426,7 +426,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G3"/>
+  <dimension ref="A1:G4"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="15" customWidth="1" min="1" max="1"/>
@@ -549,6 +549,43 @@
         </is>
       </c>
     </row>
+    <row r="4">
+      <c r="A4" t="inlineStr">
+        <is>
+          <t>Player-123456</t>
+        </is>
+      </c>
+      <c r="B4" t="inlineStr">
+        <is>
+          <t>123456</t>
+        </is>
+      </c>
+      <c r="C4" t="inlineStr">
+        <is>
+          <t>****3456</t>
+        </is>
+      </c>
+      <c r="D4" t="inlineStr">
+        <is>
+          <t>0/10</t>
+        </is>
+      </c>
+      <c r="E4" t="inlineStr">
+        <is>
+          <t>0.00%</t>
+        </is>
+      </c>
+      <c r="F4" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="G4" t="inlineStr">
+        <is>
+          <t>2025-10-29 04:59:41</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Update quiz results spreadsheet
Update quiz_results.xlsx with new data.

Replit-Commit-Author: Agent
Replit-Commit-Session-Id: 37877615-d133-4c1f-b6b6-f54cbc6b3767
Replit-Commit-Checkpoint-Type: full_checkpoint
Replit-Commit-Screenshot-Url: https://storage.googleapis.com/screenshot-production-us-central1/474f6d33-5530-4c51-8e53-e2d7cdb3d75e/37877615-d133-4c1f-b6b6-f54cbc6b3767/i6VO5ei
</commit_message>
<xml_diff>
--- a/quiz_results.xlsx
+++ b/quiz_results.xlsx
@@ -426,7 +426,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G4"/>
+  <dimension ref="A1:G5"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="15" customWidth="1" min="1" max="1"/>
@@ -586,6 +586,43 @@
         </is>
       </c>
     </row>
+    <row r="5">
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>Player-123456</t>
+        </is>
+      </c>
+      <c r="B5" t="inlineStr">
+        <is>
+          <t>123456</t>
+        </is>
+      </c>
+      <c r="C5" t="inlineStr">
+        <is>
+          <t>****3456</t>
+        </is>
+      </c>
+      <c r="D5" t="inlineStr">
+        <is>
+          <t>4/10</t>
+        </is>
+      </c>
+      <c r="E5" t="inlineStr">
+        <is>
+          <t>40.00%</t>
+        </is>
+      </c>
+      <c r="F5" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="G5" t="inlineStr">
+        <is>
+          <t>2025-10-29 05:07:30</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Adjust layout and appearance of result page elements
Update styling for the "Thank You!" message, "Next" button, and prize icon on the result page.

Replit-Commit-Author: Agent
Replit-Commit-Session-Id: 37877615-d133-4c1f-b6b6-f54cbc6b3767
Replit-Commit-Checkpoint-Type: full_checkpoint
Replit-Commit-Screenshot-Url: https://storage.googleapis.com/screenshot-production-us-central1/474f6d33-5530-4c51-8e53-e2d7cdb3d75e/37877615-d133-4c1f-b6b6-f54cbc6b3767/crcJubj
</commit_message>
<xml_diff>
--- a/quiz_results.xlsx
+++ b/quiz_results.xlsx
@@ -426,7 +426,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G2"/>
+  <dimension ref="A1:G3"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="15" customWidth="1" min="1" max="1"/>
@@ -512,6 +512,43 @@
         </is>
       </c>
     </row>
+    <row r="3">
+      <c r="A3" t="inlineStr">
+        <is>
+          <t>Player-123456</t>
+        </is>
+      </c>
+      <c r="B3" t="inlineStr">
+        <is>
+          <t>123456</t>
+        </is>
+      </c>
+      <c r="C3" t="inlineStr">
+        <is>
+          <t>****3456</t>
+        </is>
+      </c>
+      <c r="D3" t="inlineStr">
+        <is>
+          <t>8/10</t>
+        </is>
+      </c>
+      <c r="E3" t="inlineStr">
+        <is>
+          <t>80.00%</t>
+        </is>
+      </c>
+      <c r="F3" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="G3" t="inlineStr">
+        <is>
+          <t>2025-10-29 05:50:48</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Adjust score display proportions on the results page
Update the result.html template and CSS to resize score text, reposition the percentage display, and adjust margin for the "Right Answers!" label.

Replit-Commit-Author: Agent
Replit-Commit-Session-Id: 37877615-d133-4c1f-b6b6-f54cbc6b3767
Replit-Commit-Checkpoint-Type: full_checkpoint
Replit-Commit-Screenshot-Url: https://storage.googleapis.com/screenshot-production-us-central1/474f6d33-5530-4c51-8e53-e2d7cdb3d75e/37877615-d133-4c1f-b6b6-f54cbc6b3767/Mhc338A
</commit_message>
<xml_diff>
--- a/quiz_results.xlsx
+++ b/quiz_results.xlsx
@@ -426,7 +426,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G3"/>
+  <dimension ref="A1:G4"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="15" customWidth="1" min="1" max="1"/>
@@ -549,6 +549,43 @@
         </is>
       </c>
     </row>
+    <row r="4">
+      <c r="A4" t="inlineStr">
+        <is>
+          <t>Player-123456</t>
+        </is>
+      </c>
+      <c r="B4" t="inlineStr">
+        <is>
+          <t>123456</t>
+        </is>
+      </c>
+      <c r="C4" t="inlineStr">
+        <is>
+          <t>****3456</t>
+        </is>
+      </c>
+      <c r="D4" t="inlineStr">
+        <is>
+          <t>8/10</t>
+        </is>
+      </c>
+      <c r="E4" t="inlineStr">
+        <is>
+          <t>80.00%</t>
+        </is>
+      </c>
+      <c r="F4" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="G4" t="inlineStr">
+        <is>
+          <t>2025-10-29 05:58:32</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>